<commit_message>
FIX[parser]: Correct parenthesys in compare cases
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/FILTER_ERRORS.xlsx
+++ b/xlsx/tests/calc_tests/LOOKUP_AND_REFERENCE/FILTER_ERRORS.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/MATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{826603CF-2BC8-E548-8240-8E7EE9E5768C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585E1AEE-B660-3B44-9241-F4EA4CBF5F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" xr2:uid="{CF0CE628-641F-7343-A6D3-5846A25FA48A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -76,9 +76,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="8">
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Calc</t>
+  </si>
+  <si>
+    <t>HR</t>
   </si>
 </sst>
 </file>
@@ -508,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D711322B-9675-4641-9620-62AEEA86E7BE}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -561,6 +582,64 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="str" cm="1">
+        <f t="array" ref="E9:E11">_xlfn._xlws.FILTER(A9:A12,(B9:B12="Finance")+(C9:C12="HR"))</f>
+        <v>a</v>
+      </c>
+      <c r="F9" t="str" cm="1">
+        <f t="array" ref="F9">_xlfn._xlws.FILTER(A9:A12,(B9:B12="Finance")*(C9:C12="HR"))</f>
+        <v>a</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="str">
+        <v>b</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" t="str">
+        <v>c</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>